<commit_message>
New template for excel deliveries
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/DeliveryTemplate.xlsx
+++ b/srv/xlsx-templates/DeliveryTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slynx\Documents\Projecten\Bayer\fastCAP_v2\fastCAP-backend\srv\xlsx-templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projects\Bayer\fastCAPv2\fastCAP-backend\srv\xlsx-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECA8B6C-960E-4BF2-B4B6-EF3A30C403B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06D124E-DFF7-4D65-8842-B728794380D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
-  <si>
-    <t>Header with Bayer Logo</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>${offerValidation.INSTITUTENAME}</t>
   </si>
@@ -152,7 +149,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -167,8 +164,242 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>554182</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>65463</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="7" name="Group 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28F130C5-50B4-4785-AADD-D21FE0A17F6A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="24588008" cy="1102649"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="12852400" cy="573002"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="Oval 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2255F03B-25EF-4116-A24E-1C33ED4569A5}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks noChangeAspect="1"/>
+          </xdr:cNvSpPr>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="12141200" y="0"/>
+            <a:ext cx="711200" cy="573002"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="10384F"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="9" name="Rectangle 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB2893E6-F0FC-4EF4-9B62-A50EC91E664F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="12520901" cy="573002"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="10384F"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="2800" b="1"/>
+              <a:t>		FAST Deliveries Extract</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="10" name="Graphic 9">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D32CD9F8-E5A5-4D50-8A58-9A7702B05E1C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+              <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="63293" y="15916"/>
+            <a:ext cx="622766" cy="547536"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="11" name="Picture 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12CD7B93-7F0A-4ACC-9798-6405014926EC}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="11488971" y="26619"/>
+            <a:ext cx="1132381" cy="522734"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="10384F"/>
+          </a:solidFill>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -464,118 +695,114 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F4731A-D70B-4034-AE07-DF495FD0B95B}">
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A10:L14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="27" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
         <v>3</v>
       </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
+        <v>10</v>
+      </c>
+      <c r="J13" t="s">
+        <v>11</v>
+      </c>
+      <c r="K13" t="s">
+        <v>12</v>
+      </c>
+      <c r="L13" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6" t="s">
-        <v>10</v>
-      </c>
-      <c r="I6" t="s">
-        <v>11</v>
-      </c>
-      <c r="J6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K6" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6" t="s">
+      <c r="B14" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="C14" t="s">
         <v>17</v>
       </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E14" t="s">
         <v>19</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G14" t="s">
         <v>21</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H14" t="s">
         <v>22</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I14" t="s">
         <v>23</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J14" t="s">
         <v>24</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K14" t="s">
         <v>25</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L14" t="s">
         <v>26</v>
-      </c>
-      <c r="L7" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Deliveries not returning all data in excel
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/DeliveryTemplate.xlsx
+++ b/srv/xlsx-templates/DeliveryTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projects\Bayer\fastCAPv2\fastCAP-backend\srv\xlsx-templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slynx\Documents\Projecten\Bayer\fastCAP_v2\fastCAP-backend\srv\xlsx-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06D124E-DFF7-4D65-8842-B728794380D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E585B41E-8C4E-4651-BB42-9BA483D1F4D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>${offerValidation.INSTITUTENAME}</t>
   </si>
@@ -106,6 +106,18 @@
   </si>
   <si>
     <t>${table:deliveries.Compensated}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFFER ID </t>
+  </si>
+  <si>
+    <t>${offerValidation.OFFERID}</t>
+  </si>
+  <si>
+    <t>PRODUCT NAME</t>
+  </si>
+  <si>
+    <t>${table:deliveries.ProductName}</t>
   </si>
 </sst>
 </file>
@@ -149,7 +161,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -174,7 +186,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>554182</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>65463</xdr:rowOff>
@@ -193,7 +205,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="24588008" cy="1102649"/>
+          <a:ext cx="26550105" cy="1208463"/>
           <a:chOff x="0" y="0"/>
           <a:chExt cx="12852400" cy="573002"/>
         </a:xfrm>
@@ -399,7 +411,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -695,23 +707,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F4731A-D70B-4034-AE07-DF495FD0B95B}">
-  <dimension ref="A10:L14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A9:M14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -719,84 +740,90 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
       <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
         <v>3</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>4</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>5</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>6</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>7</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>8</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>9</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>10</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>11</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>12</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
         <v>14</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>21</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>22</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>23</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>24</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>25</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>